<commit_message>
Session dates: Session 01 on Oct 21, Session 02 on Oct 28, 2026; drop calendar-link requests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0123W63ZaDAAnYHCFqarTnbL
</commit_message>
<xml_diff>
--- a/Building Agentic Platforms - programme.xlsx
+++ b/Building Agentic Platforms - programme.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Programme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sessions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sessions'!$A$1:$M$13</definedName>
@@ -488,7 +488,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>